<commit_message>
refined fuel, technology, and portfolio data
</commit_message>
<xml_diff>
--- a/data/_master-data/fuel data.xlsx
+++ b/data/_master-data/fuel data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jujmo\Github\J4\data\_master-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C469E0-8877-40E9-84B2-EDC47D375D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EFBFAB5-9DF9-4C10-BD5A-9906F5E10171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43200" yWindow="450" windowWidth="14400" windowHeight="17550" activeTab="1" xr2:uid="{6E05FBF9-7A0C-4B38-8AD0-297E8124D7D0}"/>
+    <workbookView xWindow="28680" yWindow="330" windowWidth="29040" windowHeight="17790" activeTab="1" xr2:uid="{6E05FBF9-7A0C-4B38-8AD0-297E8124D7D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="68">
   <si>
     <t>name</t>
   </si>
@@ -245,6 +245,9 @@
   </si>
   <si>
     <t>Total tax</t>
+  </si>
+  <si>
+    <t>Total cost</t>
   </si>
 </sst>
 </file>
@@ -384,16 +387,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3252,7 +3255,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{931181A0-02B4-4BE8-AAB8-3DB7EDEE65B2}">
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.7265625" bestFit="1" customWidth="1"/>
@@ -3260,9 +3263,10 @@
     <col min="8" max="12" width="10.7265625" customWidth="1"/>
     <col min="13" max="14" width="10.453125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>30</v>
       </c>
@@ -3273,7 +3277,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -3284,7 +3288,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>63</v>
       </c>
@@ -3295,31 +3299,31 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B4" s="6"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="B5" s="20" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="B5" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21" t="s">
+      <c r="C5" s="22"/>
+      <c r="D5" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21" t="s">
+      <c r="E5" s="23"/>
+      <c r="F5" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="G5" s="21"/>
-      <c r="H5" s="21" t="s">
+      <c r="G5" s="23"/>
+      <c r="H5" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21" t="s">
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="21"/>
+      <c r="L5" s="23"/>
       <c r="M5" s="19" t="s">
         <v>53</v>
       </c>
@@ -3329,8 +3333,11 @@
       <c r="O5" s="19" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="P5" s="19" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="16"/>
       <c r="B6" s="13" t="s">
         <v>18</v>
@@ -3375,7 +3382,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
         <v>6</v>
       </c>
@@ -3416,7 +3423,7 @@
       <c r="L7" t="s">
         <v>59</v>
       </c>
-      <c r="M7" s="23">
+      <c r="M7" s="21">
         <f>H7*(1/K7)*$B$2*$B$1</f>
         <v>1.1947090909090907</v>
       </c>
@@ -3428,8 +3435,12 @@
         <f>M7+N7</f>
         <v>1.1947090909090907</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P7" s="7">
+        <f>C7+O7+E7*G7</f>
+        <v>81.590043712551548</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
         <v>12</v>
       </c>
@@ -3481,8 +3492,12 @@
         <f t="shared" ref="O8:O17" si="3">M8+N8</f>
         <v>35.482860000000002</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P8" s="7">
+        <f t="shared" ref="P8:P17" si="4">C8+O8+E8*G8</f>
+        <v>52.257949480754391</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
         <v>14</v>
       </c>
@@ -3501,7 +3516,7 @@
       <c r="F9">
         <v>175</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="20">
         <f t="shared" si="2"/>
         <v>2.3467500000000002E-2</v>
       </c>
@@ -3532,8 +3547,12 @@
         <f t="shared" si="3"/>
         <v>11.96172</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P9" s="7" t="e">
+        <f t="shared" si="4"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
         <v>16</v>
       </c>
@@ -3583,8 +3602,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P10" s="7">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
         <v>10</v>
       </c>
@@ -3636,8 +3659,12 @@
         <f t="shared" si="3"/>
         <v>34.048534317343169</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P11" s="7">
+        <f t="shared" si="4"/>
+        <v>70.339035219790446</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
         <v>11</v>
       </c>
@@ -3689,8 +3716,12 @@
         <f t="shared" si="3"/>
         <v>33.702214787554361</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P12" s="7">
+        <f t="shared" si="4"/>
+        <v>87.181160687554367</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="12" t="s">
         <v>13</v>
       </c>
@@ -3740,8 +3771,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P13" s="7">
+        <f t="shared" si="4"/>
+        <v>-16.106080499999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="12" t="s">
         <v>7</v>
       </c>
@@ -3794,8 +3829,12 @@
         <f t="shared" si="3"/>
         <v>32.265293255872692</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P14" s="7">
+        <f t="shared" si="4"/>
+        <v>58.766277682350221</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="12" t="s">
         <v>9</v>
       </c>
@@ -3845,8 +3884,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P15" s="7">
+        <f t="shared" si="4"/>
+        <v>25.8614532</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="12" t="s">
         <v>8</v>
       </c>
@@ -3896,8 +3939,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="P16" s="7">
+        <f t="shared" si="4"/>
+        <v>34.918030800000004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="14" t="s">
         <v>15</v>
       </c>
@@ -3946,6 +3993,10 @@
       <c r="O17" s="18">
         <f t="shared" si="3"/>
         <v>0</v>
+      </c>
+      <c r="P17" s="7">
+        <f t="shared" si="4"/>
+        <v>12.069000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>